<commit_message>
Real end-to-end compiler run from certified canonical state (80fba4d)
python3 -m compiler.run_compiler executed against commit 80fba4d;
full pytest suite (720 tests) and compiler/tests (141 tests) both green.
All 10 self-audits PASS, terminal status CONDITIONALLY_CLOSED.
status_matrix.json, proof_registry.json, chainlink_registry.json,
self_audit_report.json, target_independence.json bitwise-identical to
pre-run state, independently confirming numerical_reproducibility_audit.
Remaining diffs are execution_timestamp/git_commit/run_timestamp fields
only -- zero semantic drift.
</commit_message>
<xml_diff>
--- a/Master Calculation Workbook.xlsx
+++ b/Master Calculation Workbook.xlsx
@@ -1670,12 +1670,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.154621+00:00</t>
+          <t>2026-08-21T20:17:14.864356+00:00</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1697,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.157123+00:00</t>
+          <t>2026-08-21T20:17:14.866689+00:00</t>
         </is>
       </c>
     </row>
@@ -1724,12 +1724,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.159525+00:00</t>
+          <t>2026-08-21T20:17:14.868765+00:00</t>
         </is>
       </c>
     </row>
@@ -1751,12 +1751,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.161801+00:00</t>
+          <t>2026-08-21T20:17:14.870877+00:00</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1778,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.163720+00:00</t>
+          <t>2026-08-21T20:17:14.872890+00:00</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.166106+00:00</t>
+          <t>2026-08-21T20:17:14.874907+00:00</t>
         </is>
       </c>
     </row>
@@ -1832,12 +1832,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.168374+00:00</t>
+          <t>2026-08-21T20:17:14.876820+00:00</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1859,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.170531+00:00</t>
+          <t>2026-08-21T20:17:14.878925+00:00</t>
         </is>
       </c>
     </row>
@@ -1886,12 +1886,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.172495+00:00</t>
+          <t>2026-08-21T20:17:14.880978+00:00</t>
         </is>
       </c>
     </row>
@@ -1913,12 +1913,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.174611+00:00</t>
+          <t>2026-08-21T20:17:14.882989+00:00</t>
         </is>
       </c>
     </row>
@@ -1940,12 +1940,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.176467+00:00</t>
+          <t>2026-08-21T20:17:14.884960+00:00</t>
         </is>
       </c>
     </row>
@@ -1967,12 +1967,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.178859+00:00</t>
+          <t>2026-08-21T20:17:14.887056+00:00</t>
         </is>
       </c>
     </row>
@@ -1994,12 +1994,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.181148+00:00</t>
+          <t>2026-08-21T20:17:14.888924+00:00</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.183253+00:00</t>
+          <t>2026-08-21T20:17:14.891004+00:00</t>
         </is>
       </c>
     </row>
@@ -2048,12 +2048,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.185062+00:00</t>
+          <t>2026-08-21T20:17:14.892894+00:00</t>
         </is>
       </c>
     </row>
@@ -2075,12 +2075,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.187573+00:00</t>
+          <t>2026-08-21T20:17:14.894819+00:00</t>
         </is>
       </c>
     </row>
@@ -2102,12 +2102,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.189525+00:00</t>
+          <t>2026-08-21T20:17:14.896625+00:00</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.192047+00:00</t>
+          <t>2026-08-21T20:17:14.898419+00:00</t>
         </is>
       </c>
     </row>
@@ -2156,12 +2156,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.194073+00:00</t>
+          <t>2026-08-21T20:17:14.900221+00:00</t>
         </is>
       </c>
     </row>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.195966+00:00</t>
+          <t>2026-08-21T20:17:14.902239+00:00</t>
         </is>
       </c>
     </row>
@@ -2210,12 +2210,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.198190+00:00</t>
+          <t>2026-08-21T20:17:14.904040+00:00</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.432408+00:00</t>
+          <t>2026-08-21T20:17:15.014910+00:00</t>
         </is>
       </c>
     </row>
@@ -2264,12 +2264,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.436828+00:00</t>
+          <t>2026-08-21T20:17:15.017273+00:00</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2291,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.440005+00:00</t>
+          <t>2026-08-21T20:17:15.019361+00:00</t>
         </is>
       </c>
     </row>
@@ -2318,12 +2318,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.443962+00:00</t>
+          <t>2026-08-21T20:17:15.021290+00:00</t>
         </is>
       </c>
     </row>
@@ -2345,12 +2345,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.632841+00:00</t>
+          <t>2026-08-21T20:17:15.216318+00:00</t>
         </is>
       </c>
     </row>
@@ -2372,12 +2372,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.635451+00:00</t>
+          <t>2026-08-21T20:17:15.219157+00:00</t>
         </is>
       </c>
     </row>
@@ -2399,12 +2399,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.066772+00:00</t>
+          <t>2026-08-21T20:17:15.637115+00:00</t>
         </is>
       </c>
     </row>
@@ -2426,12 +2426,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.471460+00:00</t>
+          <t>2026-08-21T20:17:16.052301+00:00</t>
         </is>
       </c>
     </row>
@@ -2453,12 +2453,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.473985+00:00</t>
+          <t>2026-08-21T20:17:16.054794+00:00</t>
         </is>
       </c>
     </row>
@@ -2480,12 +2480,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.476060+00:00</t>
+          <t>2026-08-21T20:17:16.056849+00:00</t>
         </is>
       </c>
     </row>
@@ -2507,12 +2507,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.478109+00:00</t>
+          <t>2026-08-21T20:17:16.058766+00:00</t>
         </is>
       </c>
     </row>
@@ -2534,12 +2534,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.480101+00:00</t>
+          <t>2026-08-21T20:17:16.060609+00:00</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.482048+00:00</t>
+          <t>2026-08-21T20:17:16.062534+00:00</t>
         </is>
       </c>
     </row>
@@ -2588,12 +2588,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.483844+00:00</t>
+          <t>2026-08-21T20:17:16.064599+00:00</t>
         </is>
       </c>
     </row>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.485738+00:00</t>
+          <t>2026-08-21T20:17:16.066589+00:00</t>
         </is>
       </c>
     </row>
@@ -2642,12 +2642,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.487570+00:00</t>
+          <t>2026-08-21T20:17:16.068477+00:00</t>
         </is>
       </c>
     </row>
@@ -2669,12 +2669,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.489391+00:00</t>
+          <t>2026-08-21T20:17:16.070367+00:00</t>
         </is>
       </c>
     </row>
@@ -2696,12 +2696,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.629195+00:00</t>
+          <t>2026-08-21T20:17:16.211781+00:00</t>
         </is>
       </c>
     </row>
@@ -2723,12 +2723,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.631220+00:00</t>
+          <t>2026-08-21T20:17:16.213677+00:00</t>
         </is>
       </c>
     </row>
@@ -2750,12 +2750,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.633173+00:00</t>
+          <t>2026-08-21T20:17:16.215621+00:00</t>
         </is>
       </c>
     </row>
@@ -2777,12 +2777,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.635082+00:00</t>
+          <t>2026-08-21T20:17:16.217664+00:00</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.636805+00:00</t>
+          <t>2026-08-21T20:17:16.219469+00:00</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2831,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.385367+00:00</t>
+          <t>2026-08-21T20:17:18.172147+00:00</t>
         </is>
       </c>
     </row>
@@ -2858,12 +2858,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.388048+00:00</t>
+          <t>2026-08-21T20:17:18.175341+00:00</t>
         </is>
       </c>
     </row>
@@ -2885,12 +2885,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.391857+00:00</t>
+          <t>2026-08-21T20:17:18.179062+00:00</t>
         </is>
       </c>
     </row>
@@ -2912,12 +2912,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.396343+00:00</t>
+          <t>2026-08-21T20:17:18.183045+00:00</t>
         </is>
       </c>
     </row>
@@ -2939,12 +2939,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.402130+00:00</t>
+          <t>2026-08-21T20:17:18.189477+00:00</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.404894+00:00</t>
+          <t>2026-08-21T20:17:18.191528+00:00</t>
         </is>
       </c>
     </row>
@@ -2993,12 +2993,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.408060+00:00</t>
+          <t>2026-08-21T20:17:18.195175+00:00</t>
         </is>
       </c>
     </row>
@@ -3020,12 +3020,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.411713+00:00</t>
+          <t>2026-08-21T20:17:18.201548+00:00</t>
         </is>
       </c>
     </row>
@@ -3047,12 +3047,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.418148+00:00</t>
+          <t>2026-08-21T20:17:18.203798+00:00</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3074,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.420090+00:00</t>
+          <t>2026-08-21T20:17:18.207336+00:00</t>
         </is>
       </c>
     </row>
@@ -3101,12 +3101,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.426071+00:00</t>
+          <t>2026-08-21T20:17:18.213524+00:00</t>
         </is>
       </c>
     </row>
@@ -3128,12 +3128,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.427985+00:00</t>
+          <t>2026-08-21T20:17:18.217542+00:00</t>
         </is>
       </c>
     </row>
@@ -3155,12 +3155,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.434088+00:00</t>
+          <t>2026-08-21T20:17:18.223058+00:00</t>
         </is>
       </c>
     </row>
@@ -3182,12 +3182,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.436177+00:00</t>
+          <t>2026-08-21T20:17:18.227128+00:00</t>
         </is>
       </c>
     </row>
@@ -3209,12 +3209,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.439617+00:00</t>
+          <t>2026-08-21T20:17:18.233454+00:00</t>
         </is>
       </c>
     </row>
@@ -3236,12 +3236,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.860520+00:00</t>
+          <t>2026-08-21T20:17:18.686893+00:00</t>
         </is>
       </c>
     </row>
@@ -3263,12 +3263,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.871089+00:00</t>
+          <t>2026-08-21T20:17:18.697736+00:00</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3290,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.875076+00:00</t>
+          <t>2026-08-21T20:17:18.701746+00:00</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3317,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.882142+00:00</t>
+          <t>2026-08-21T20:17:18.709058+00:00</t>
         </is>
       </c>
     </row>
@@ -3344,12 +3344,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.888017+00:00</t>
+          <t>2026-08-21T20:17:18.715380+00:00</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3371,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.895714+00:00</t>
+          <t>2026-08-21T20:17:18.723052+00:00</t>
         </is>
       </c>
     </row>
@@ -3398,12 +3398,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.902105+00:00</t>
+          <t>2026-08-21T20:17:18.729498+00:00</t>
         </is>
       </c>
     </row>
@@ -3425,12 +3425,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.904323+00:00</t>
+          <t>2026-08-21T20:17:18.731370+00:00</t>
         </is>
       </c>
     </row>
@@ -3452,12 +3452,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:01.171465+00:00</t>
+          <t>2026-08-21T20:17:19.016556+00:00</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.128754+00:00</t>
+          <t>2026-08-21T20:17:25.075472+00:00</t>
         </is>
       </c>
     </row>
@@ -3506,12 +3506,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.133963+00:00</t>
+          <t>2026-08-21T20:17:25.080610+00:00</t>
         </is>
       </c>
     </row>
@@ -3533,12 +3533,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.141103+00:00</t>
+          <t>2026-08-21T20:17:25.088437+00:00</t>
         </is>
       </c>
     </row>
@@ -3560,12 +3560,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.145110+00:00</t>
+          <t>2026-08-21T20:17:25.092476+00:00</t>
         </is>
       </c>
     </row>
@@ -3587,12 +3587,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.147141+00:00</t>
+          <t>2026-08-21T20:17:25.094764+00:00</t>
         </is>
       </c>
     </row>
@@ -3614,12 +3614,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.148904+00:00</t>
+          <t>2026-08-21T20:17:25.096728+00:00</t>
         </is>
       </c>
     </row>
@@ -3641,12 +3641,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.150744+00:00</t>
+          <t>2026-08-21T20:17:25.098586+00:00</t>
         </is>
       </c>
     </row>
@@ -3668,12 +3668,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.152492+00:00</t>
+          <t>2026-08-21T20:17:25.100987+00:00</t>
         </is>
       </c>
     </row>
@@ -3695,12 +3695,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.154399+00:00</t>
+          <t>2026-08-21T20:17:25.103014+00:00</t>
         </is>
       </c>
     </row>
@@ -3722,12 +3722,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.156200+00:00</t>
+          <t>2026-08-21T20:17:25.105016+00:00</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.347476+00:00</t>
+          <t>2026-08-21T20:17:25.252148+00:00</t>
         </is>
       </c>
     </row>
@@ -3776,12 +3776,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.350591+00:00</t>
+          <t>2026-08-21T20:17:25.255367+00:00</t>
         </is>
       </c>
     </row>
@@ -3803,12 +3803,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.355692+00:00</t>
+          <t>2026-08-21T20:17:25.259093+00:00</t>
         </is>
       </c>
     </row>
@@ -3830,12 +3830,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.359716+00:00</t>
+          <t>2026-08-21T20:17:25.263058+00:00</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.368019+00:00</t>
+          <t>2026-08-21T20:17:25.271033+00:00</t>
         </is>
       </c>
     </row>
@@ -3884,12 +3884,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.418159+00:00</t>
+          <t>2026-08-21T20:17:25.319636+00:00</t>
         </is>
       </c>
     </row>
@@ -3911,12 +3911,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.421987+00:00</t>
+          <t>2026-08-21T20:17:25.322088+00:00</t>
         </is>
       </c>
     </row>
@@ -3938,12 +3938,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.423967+00:00</t>
+          <t>2026-08-21T20:17:25.327160+00:00</t>
         </is>
       </c>
     </row>
@@ -3965,12 +3965,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.427644+00:00</t>
+          <t>2026-08-21T20:17:25.331118+00:00</t>
         </is>
       </c>
     </row>
@@ -3992,12 +3992,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.435543+00:00</t>
+          <t>2026-08-21T20:17:25.339378+00:00</t>
         </is>
       </c>
     </row>
@@ -4019,12 +4019,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.439494+00:00</t>
+          <t>2026-08-21T20:17:25.341526+00:00</t>
         </is>
       </c>
     </row>
@@ -4046,12 +4046,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.280124+00:00</t>
+          <t>2026-08-21T20:17:27.314290+00:00</t>
         </is>
       </c>
     </row>
@@ -4073,12 +4073,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.282484+00:00</t>
+          <t>2026-08-21T20:17:27.319765+00:00</t>
         </is>
       </c>
     </row>
@@ -4100,12 +4100,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.287791+00:00</t>
+          <t>2026-08-21T20:17:27.323036+00:00</t>
         </is>
       </c>
     </row>
@@ -4127,12 +4127,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.291706+00:00</t>
+          <t>2026-08-21T20:17:27.327019+00:00</t>
         </is>
       </c>
     </row>
@@ -4154,12 +4154,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.293600+00:00</t>
+          <t>2026-08-21T20:17:27.330958+00:00</t>
         </is>
       </c>
     </row>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.295575+00:00</t>
+          <t>2026-08-21T20:17:27.335092+00:00</t>
         </is>
       </c>
     </row>
@@ -4208,12 +4208,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.739288+00:00</t>
+          <t>2026-08-21T20:17:27.775915+00:00</t>
         </is>
       </c>
     </row>
@@ -4235,12 +4235,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:17.188222+00:00</t>
+          <t>2026-08-21T20:17:34.874428+00:00</t>
         </is>
       </c>
     </row>
@@ -4262,12 +4262,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:17.191957+00:00</t>
+          <t>2026-08-21T20:17:34.876751+00:00</t>
         </is>
       </c>
     </row>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:17.200602+00:00</t>
+          <t>2026-08-21T20:17:34.880386+00:00</t>
         </is>
       </c>
     </row>
@@ -4316,12 +4316,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.151479+00:00</t>
+          <t>2026-08-21T20:17:14.861822+00:00</t>
         </is>
       </c>
     </row>
@@ -4343,12 +4343,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.447746+00:00</t>
+          <t>2026-08-21T20:17:15.023230+00:00</t>
         </is>
       </c>
     </row>
@@ -4370,12 +4370,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.451731+00:00</t>
+          <t>2026-08-21T20:17:15.025127+00:00</t>
         </is>
       </c>
     </row>
@@ -4397,12 +4397,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.455650+00:00</t>
+          <t>2026-08-21T20:17:15.027145+00:00</t>
         </is>
       </c>
     </row>
@@ -4424,12 +4424,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.462097+00:00</t>
+          <t>2026-08-21T20:17:15.029023+00:00</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4451,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.640022+00:00</t>
+          <t>2026-08-21T20:17:15.223223+00:00</t>
         </is>
       </c>
     </row>
@@ -4478,12 +4478,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.643859+00:00</t>
+          <t>2026-08-21T20:17:15.227376+00:00</t>
         </is>
       </c>
     </row>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.069495+00:00</t>
+          <t>2026-08-21T20:17:15.640401+00:00</t>
         </is>
       </c>
     </row>
@@ -4532,12 +4532,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.640334+00:00</t>
+          <t>2026-08-21T20:17:16.223323+00:00</t>
         </is>
       </c>
     </row>
@@ -4559,12 +4559,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:01.173954+00:00</t>
+          <t>2026-08-21T20:17:19.018932+00:00</t>
         </is>
       </c>
     </row>
@@ -4586,12 +4586,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.131397+00:00</t>
+          <t>2026-08-21T20:17:25.078422+00:00</t>
         </is>
       </c>
     </row>
@@ -4613,12 +4613,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.143226+00:00</t>
+          <t>2026-08-21T20:17:25.090619+00:00</t>
         </is>
       </c>
     </row>
@@ -4640,12 +4640,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.366107+00:00</t>
+          <t>2026-08-21T20:17:25.267043+00:00</t>
         </is>
       </c>
     </row>
@@ -4667,12 +4667,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:07.430977+00:00</t>
+          <t>2026-08-21T20:17:25.337497+00:00</t>
         </is>
       </c>
     </row>
@@ -4694,12 +4694,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.299578+00:00</t>
+          <t>2026-08-21T20:17:27.336880+00:00</t>
         </is>
       </c>
     </row>
@@ -4721,12 +4721,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:09.741613+00:00</t>
+          <t>2026-08-21T20:17:27.778387+00:00</t>
         </is>
       </c>
     </row>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:17.195672+00:00</t>
+          <t>2026-08-21T20:17:34.878649+00:00</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4775,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.651985+00:00</t>
+          <t>2026-08-21T20:17:15.241935+00:00</t>
         </is>
       </c>
     </row>
@@ -4802,12 +4802,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:56.654658+00:00</t>
+          <t>2026-08-21T20:17:15.244013+00:00</t>
         </is>
       </c>
     </row>
@@ -4829,12 +4829,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.560199+00:00</t>
+          <t>2026-08-21T20:17:16.146768+00:00</t>
         </is>
       </c>
     </row>
@@ -4856,12 +4856,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.562913+00:00</t>
+          <t>2026-08-21T20:17:16.149042+00:00</t>
         </is>
       </c>
     </row>
@@ -4883,12 +4883,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.565141+00:00</t>
+          <t>2026-08-21T20:17:16.151116+00:00</t>
         </is>
       </c>
     </row>
@@ -4910,12 +4910,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.567230+00:00</t>
+          <t>2026-08-21T20:17:16.153015+00:00</t>
         </is>
       </c>
     </row>
@@ -4937,12 +4937,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.569206+00:00</t>
+          <t>2026-08-21T20:17:16.155064+00:00</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.571333+00:00</t>
+          <t>2026-08-21T20:17:16.157111+00:00</t>
         </is>
       </c>
     </row>
@@ -4991,12 +4991,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.573357+00:00</t>
+          <t>2026-08-21T20:17:16.158997+00:00</t>
         </is>
       </c>
     </row>
@@ -5018,12 +5018,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.575503+00:00</t>
+          <t>2026-08-21T20:17:16.160990+00:00</t>
         </is>
       </c>
     </row>
@@ -5045,12 +5045,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.577332+00:00</t>
+          <t>2026-08-21T20:17:16.162892+00:00</t>
         </is>
       </c>
     </row>
@@ -5072,12 +5072,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.579253+00:00</t>
+          <t>2026-08-21T20:17:16.165127+00:00</t>
         </is>
       </c>
     </row>
@@ -5099,12 +5099,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.581275+00:00</t>
+          <t>2026-08-21T20:17:16.167395+00:00</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5126,12 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.583250+00:00</t>
+          <t>2026-08-21T20:17:16.169370+00:00</t>
         </is>
       </c>
     </row>
@@ -5153,12 +5153,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.585149+00:00</t>
+          <t>2026-08-21T20:17:16.171721+00:00</t>
         </is>
       </c>
     </row>
@@ -5180,12 +5180,12 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.587068+00:00</t>
+          <t>2026-08-21T20:17:16.173737+00:00</t>
         </is>
       </c>
     </row>
@@ -5207,12 +5207,12 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.588870+00:00</t>
+          <t>2026-08-21T20:17:16.175853+00:00</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5234,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.590814+00:00</t>
+          <t>2026-08-21T20:17:16.177846+00:00</t>
         </is>
       </c>
     </row>
@@ -5261,12 +5261,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.592647+00:00</t>
+          <t>2026-08-21T20:17:16.179771+00:00</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.594744+00:00</t>
+          <t>2026-08-21T20:17:16.181988+00:00</t>
         </is>
       </c>
     </row>
@@ -5315,12 +5315,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.596736+00:00</t>
+          <t>2026-08-21T20:17:16.183757+00:00</t>
         </is>
       </c>
     </row>
@@ -5342,12 +5342,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.598965+00:00</t>
+          <t>2026-08-21T20:17:16.185678+00:00</t>
         </is>
       </c>
     </row>
@@ -5369,12 +5369,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.600875+00:00</t>
+          <t>2026-08-21T20:17:16.187503+00:00</t>
         </is>
       </c>
     </row>
@@ -5396,12 +5396,12 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.603386+00:00</t>
+          <t>2026-08-21T20:17:16.189252+00:00</t>
         </is>
       </c>
     </row>
@@ -5423,12 +5423,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.605443+00:00</t>
+          <t>2026-08-21T20:17:16.191055+00:00</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5450,12 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.607374+00:00</t>
+          <t>2026-08-21T20:17:16.192873+00:00</t>
         </is>
       </c>
     </row>
@@ -5477,12 +5477,12 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.609290+00:00</t>
+          <t>2026-08-21T20:17:16.194723+00:00</t>
         </is>
       </c>
     </row>
@@ -5504,12 +5504,12 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.611242+00:00</t>
+          <t>2026-08-21T20:17:16.196586+00:00</t>
         </is>
       </c>
     </row>
@@ -5531,12 +5531,12 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.613180+00:00</t>
+          <t>2026-08-21T20:17:16.198532+00:00</t>
         </is>
       </c>
     </row>
@@ -5558,12 +5558,12 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.615222+00:00</t>
+          <t>2026-08-21T20:17:16.200766+00:00</t>
         </is>
       </c>
     </row>
@@ -5585,12 +5585,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.617243+00:00</t>
+          <t>2026-08-21T20:17:16.202983+00:00</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5612,12 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2026-08-21T19:24:57.638574+00:00</t>
+          <t>2026-08-21T20:17:16.221488+00:00</t>
         </is>
       </c>
     </row>
@@ -5639,12 +5639,12 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.863463+00:00</t>
+          <t>2026-08-21T20:17:18.689258+00:00</t>
         </is>
       </c>
     </row>
@@ -5666,12 +5666,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.865616+00:00</t>
+          <t>2026-08-21T20:17:18.691346+00:00</t>
         </is>
       </c>
     </row>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>379096514980</t>
+          <t>80fba4db6b95</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2026-08-21T19:25:00.891760+00:00</t>
+          <t>2026-08-21T20:17:18.719065+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>